<commit_message>
removed session id from url
</commit_message>
<xml_diff>
--- a/media/form_g_schedule.xlsx
+++ b/media/form_g_schedule.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -448,11 +448,7 @@
           <t>State IRS:</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Isaac state</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -462,7 +458,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
@@ -497,74 +493,52 @@
       <c r="A6" t="n">
         <v>1</v>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>46086</v>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PROCESSING...</t>
-        </is>
+          <t>29799998-NG1126-588</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2800</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
         <v>2</v>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>46093</v>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PROCESSING...</t>
-        </is>
+          <t>2079169-NG1126-6441</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2500</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Mar-26</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>46086</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>29799998-NG1126-588</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Mar-26</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>46093</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2079169-NG1126-6441</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E10" s="1">
-        <f>SUM(E6:E9)</f>
+      <c r="E8" s="1">
+        <f>SUM(E6:E7)</f>
         <v/>
       </c>
     </row>

</xml_diff>